<commit_message>
Add exploratory factor analysis (EFA) on AI scale variables (Q19)
- New sheet '5_FactorAnalysis' in AIuse_Decisions_Analyzed.xlsx
- New Table 6 in Descriptives_Tables.docx
- 2-factor solution (parallel analysis): AI Implementation (α=.731) and Equity & Community (α=.651)
</commit_message>
<xml_diff>
--- a/Dr. Lauren Azevedo - AI/AIuse_Decisions_Analyzed.xlsx
+++ b/Dr. Lauren Azevedo - AI/AIuse_Decisions_Analyzed.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_ModeSubstituted" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_LabeledData" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Descriptives" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_FactorAnalysis" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,8 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="8">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,8 +70,42 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -119,6 +157,24 @@
         <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5E8F0"/>
+        <bgColor rgb="00D5E8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
+        <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -159,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -234,6 +290,44 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -58233,4 +58327,693 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>Exploratory Factor Analysis — AI Scale Variables (Q19_1 – Q19_10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>N = 125. Principal axis factoring with Varimax rotation. Parallel analysis (1,000 Monte Carlo iterations) indicates 2-factor solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Adequacy Tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Statistic</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="30" t="inlineStr">
+        <is>
+          <t>Bartlett's Test of Sphericity</t>
+        </is>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Chi-square</t>
+        </is>
+      </c>
+      <c r="C6" s="32" t="n">
+        <v>270.87</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr"/>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>&lt;.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Kaiser-Meyer-Olkin (KMO)</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n">
+        <v>0.628</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>Eigenvalues &amp; Parallel Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Eigenvalue</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>% Variance</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>Cumulative %</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="inlineStr">
+        <is>
+          <t>95th %ile (Random)</t>
+        </is>
+      </c>
+      <c r="F11" s="29" t="inlineStr">
+        <is>
+          <t>Retain?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="33" t="n">
+        <v>2.687</v>
+      </c>
+      <c r="C12" s="34" t="n">
+        <v>0.2686731326867313</v>
+      </c>
+      <c r="D12" s="34" t="n">
+        <v>0.2686731326867313</v>
+      </c>
+      <c r="E12" s="33" t="n">
+        <v>1.612</v>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="33" t="n">
+        <v>1.923</v>
+      </c>
+      <c r="C13" s="34" t="n">
+        <v>0.1922807719228078</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>0.4609539046095391</v>
+      </c>
+      <c r="E13" s="33" t="n">
+        <v>1.412</v>
+      </c>
+      <c r="F13" s="35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="33" t="n">
+        <v>1.055</v>
+      </c>
+      <c r="C14" s="34" t="n">
+        <v>0.1054894510548945</v>
+      </c>
+      <c r="D14" s="34" t="n">
+        <v>0.5664433556644336</v>
+      </c>
+      <c r="E14" s="33" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="F14" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="33" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="C15" s="34" t="n">
+        <v>0.1024897510248975</v>
+      </c>
+      <c r="D15" s="34" t="n">
+        <v>0.6689331066893311</v>
+      </c>
+      <c r="E15" s="33" t="n">
+        <v>1.178</v>
+      </c>
+      <c r="F15" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" s="33" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="C16" s="34" t="n">
+        <v>0.08419158084191582</v>
+      </c>
+      <c r="D16" s="34" t="n">
+        <v>0.753124687531247</v>
+      </c>
+      <c r="E16" s="33" t="n">
+        <v>1.085</v>
+      </c>
+      <c r="F16" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="33" t="n">
+        <v>0.708</v>
+      </c>
+      <c r="C17" s="34" t="n">
+        <v>0.07079292070792921</v>
+      </c>
+      <c r="D17" s="34" t="n">
+        <v>0.823917608239176</v>
+      </c>
+      <c r="E17" s="33" t="n">
+        <v>1.005</v>
+      </c>
+      <c r="F17" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" s="33" t="n">
+        <v>0.591</v>
+      </c>
+      <c r="C18" s="34" t="n">
+        <v>0.05909409059094091</v>
+      </c>
+      <c r="D18" s="34" t="n">
+        <v>0.883011698830117</v>
+      </c>
+      <c r="E18" s="33" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="F18" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" s="33" t="n">
+        <v>0.521</v>
+      </c>
+      <c r="C19" s="34" t="n">
+        <v>0.05209479052094792</v>
+      </c>
+      <c r="D19" s="34" t="n">
+        <v>0.9351064893510649</v>
+      </c>
+      <c r="E19" s="33" t="n">
+        <v>0.843</v>
+      </c>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" s="33" t="n">
+        <v>0.384</v>
+      </c>
+      <c r="C20" s="34" t="n">
+        <v>0.0383961603839616</v>
+      </c>
+      <c r="D20" s="34" t="n">
+        <v>0.9735026497350264</v>
+      </c>
+      <c r="E20" s="33" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="F20" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="33" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="C21" s="34" t="n">
+        <v>0.0264973502649735</v>
+      </c>
+      <c r="D21" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="33" t="n">
+        <v>0.679</v>
+      </c>
+      <c r="F21" s="31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>2-Factor Solution — Rotated Factor Loadings (Varimax)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>Factor 1:
+AI Implementation</t>
+        </is>
+      </c>
+      <c r="C24" s="29" t="inlineStr">
+        <is>
+          <t>Factor 2:
+Equity &amp; Community</t>
+        </is>
+      </c>
+      <c r="D24" s="29" t="inlineStr">
+        <is>
+          <t>Communality (h²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Data Quality (Q19_1)</t>
+        </is>
+      </c>
+      <c r="B25" s="36" t="n">
+        <v>0.603</v>
+      </c>
+      <c r="C25" s="33" t="n">
+        <v>-0.006</v>
+      </c>
+      <c r="D25" s="33" t="n">
+        <v>0.364</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>AI Accessibility (Q19_2)</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="n">
+        <v>0.645</v>
+      </c>
+      <c r="C26" s="33" t="n">
+        <v>0.148</v>
+      </c>
+      <c r="D26" s="33" t="n">
+        <v>0.438</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>Transparency (Q19_3)</t>
+        </is>
+      </c>
+      <c r="B27" s="33" t="n">
+        <v>-0.028</v>
+      </c>
+      <c r="C27" s="36" t="n">
+        <v>0.495</v>
+      </c>
+      <c r="D27" s="33" t="n">
+        <v>0.246</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Ethical Guidelines (Q19_4)</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="C28" s="33" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="D28" s="33" t="n">
+        <v>0.404</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Equitable Resource Dist. (Q19_5)</t>
+        </is>
+      </c>
+      <c r="B29" s="36" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="C29" s="33" t="n">
+        <v>-0.117</v>
+      </c>
+      <c r="D29" s="33" t="n">
+        <v>0.388</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Equity in Funding (Q19_6)</t>
+        </is>
+      </c>
+      <c r="B30" s="33" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="C30" s="36" t="n">
+        <v>0.742</v>
+      </c>
+      <c r="D30" s="33" t="n">
+        <v>0.576</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>AI Literacy Training (Q19_7)</t>
+        </is>
+      </c>
+      <c r="B31" s="36" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="C31" s="33" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="D31" s="33" t="n">
+        <v>0.545</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>External Resources (Q19_8)</t>
+        </is>
+      </c>
+      <c r="B32" s="33" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="C32" s="36" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="D32" s="33" t="n">
+        <v>0.796</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Community Engagement (Q19_9)</t>
+        </is>
+      </c>
+      <c r="B33" s="33" t="n">
+        <v>-0.008999999999999999</v>
+      </c>
+      <c r="C33" s="36" t="n">
+        <v>0.599</v>
+      </c>
+      <c r="D33" s="33" t="n">
+        <v>0.359</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="30" t="inlineStr">
+        <is>
+          <t>AI Expert Collaboration (Q19_10)</t>
+        </is>
+      </c>
+      <c r="B34" s="36" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="C34" s="33" t="n">
+        <v>-0.044</v>
+      </c>
+      <c r="D34" s="33" t="n">
+        <v>0.493</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="37" t="inlineStr">
+        <is>
+          <t>SS Loadings</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="n">
+        <v>2.593</v>
+      </c>
+      <c r="C35" s="38" t="n">
+        <v>2.016</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="37" t="inlineStr">
+        <is>
+          <t>Proportion of Variance</t>
+        </is>
+      </c>
+      <c r="B36" s="39" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="C36" s="39" t="n">
+        <v>0.202</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="37" t="inlineStr">
+        <is>
+          <t>Cumulative Variance</t>
+        </is>
+      </c>
+      <c r="B37" s="39" t="n">
+        <v>0.259</v>
+      </c>
+      <c r="C37" s="39" t="n">
+        <v>0.461</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="28" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>Cronbach's α</t>
+        </is>
+      </c>
+      <c r="D40" s="29" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Factor 1: AI Implementation</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t>Q19_1, Q19_2, Q19_4, Q19_5, Q19_7, Q19_10</t>
+        </is>
+      </c>
+      <c r="C41" s="33" t="n">
+        <v>0.731</v>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>Factor 2: Equity &amp; Community</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t>Q19_3, Q19_6, Q19_8, Q19_9</t>
+        </is>
+      </c>
+      <c r="C42" s="33" t="n">
+        <v>0.651</v>
+      </c>
+      <c r="D42" s="31" t="inlineStr">
+        <is>
+          <t>Questionable</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="40" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="41" t="inlineStr">
+        <is>
+          <t>Extraction: Principal axis factoring. Rotation: Varimax (orthogonal). Factor retention: Parallel analysis (95th percentile criterion, 1,000 iterations).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>Yellow-highlighted loadings ≥ |0.40| indicate primary factor membership. KMO = 0.628 (mediocre but adequate). Bartlett's test significant (p &lt; .001).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="41" t="inlineStr">
+        <is>
+          <t>Factor 1 (AI Implementation): Items related to AI infrastructure, technical capacity, and AI-specific policies. Factor 2 (Equity &amp; Community): Items related to broader equity values and stakeholder engagement.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>